<commit_message>
Keep values below 1 and refuse oversized durations
An .xlsx now reads back from its XML what the reader loses, and a duration too large gets a refusal naming its sheet and row.
</commit_message>
<xml_diff>
--- a/tests/data/synthetic-cells/cells-1900-resaved.xlsx
+++ b/tests/data/synthetic-cells/cells-1900-resaved.xlsx
@@ -559,7 +559,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L66"/>
+  <dimension ref="A1:M66"/>
   <sheetFormatPr defaultColWidth="8.5078125" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -599,6 +599,9 @@
       <c r="L1" s="1" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M1" s="1" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="n">
@@ -637,6 +640,9 @@
       <c r="L2" s="2" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M2" s="2" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="n">
@@ -675,6 +681,9 @@
       <c r="L3" s="3" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M3" s="3" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="n">
@@ -713,6 +722,9 @@
       <c r="L4" s="4" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M4" s="4" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="n">
@@ -751,6 +763,9 @@
       <c r="L5" s="5" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M5" s="5" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="n">
@@ -789,6 +804,9 @@
       <c r="L6" s="6" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M6" s="6" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="n">
@@ -827,6 +845,9 @@
       <c r="L7" s="7" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M7" s="7" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="n">
@@ -865,6 +886,9 @@
       <c r="L8" s="8" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M8" s="8" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="n">
@@ -903,6 +927,9 @@
       <c r="L9" s="9" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M9" s="9" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="n">
@@ -941,6 +968,9 @@
       <c r="L10" s="10" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M10" s="10" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="n">
@@ -979,6 +1009,9 @@
       <c r="L11" s="11" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M11" s="11" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="12" t="n">
@@ -1017,6 +1050,9 @@
       <c r="L12" s="12" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M12" s="12" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="n">
@@ -1055,6 +1091,9 @@
       <c r="L13" s="13" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M13" s="13" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="n">
@@ -1093,6 +1132,9 @@
       <c r="L14" s="14" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M14" s="14" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="15" t="n">
@@ -1131,6 +1173,9 @@
       <c r="L15" s="15" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M15" s="15" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="16" t="n">
@@ -1169,6 +1214,9 @@
       <c r="L16" s="16" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M16" s="16" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="17" t="n">
@@ -1207,6 +1255,9 @@
       <c r="L17" s="17" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M17" s="17" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="18" t="n">
@@ -1245,6 +1296,9 @@
       <c r="L18" s="18" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M18" s="18" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="19" t="n">
@@ -1283,6 +1337,9 @@
       <c r="L19" s="19" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M19" s="19" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="20" t="n">
@@ -1321,6 +1378,9 @@
       <c r="L20" s="20" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M20" s="20" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="21" t="n">
@@ -1359,6 +1419,9 @@
       <c r="L21" s="21" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M21" s="21" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="22" t="n">
@@ -1397,6 +1460,9 @@
       <c r="L22" s="22" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M22" s="22" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="23" t="n">
@@ -1435,6 +1501,9 @@
       <c r="L23" s="23" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M23" s="23" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="24" t="n">
@@ -1473,6 +1542,9 @@
       <c r="L24" s="24" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M24" s="24" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="25" t="n">
@@ -1511,6 +1583,9 @@
       <c r="L25" s="25" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M25" s="25" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="26" t="n">
@@ -1549,6 +1624,9 @@
       <c r="L26" s="26" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M26" s="26" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="27" t="n">
@@ -1587,6 +1665,9 @@
       <c r="L27" s="27" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M27" s="27" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="28" t="n">
@@ -1625,6 +1706,9 @@
       <c r="L28" s="28" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M28" s="28" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="29" t="n">
@@ -1663,6 +1747,9 @@
       <c r="L29" s="29" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M29" s="29" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="30" t="n">
@@ -1701,6 +1788,9 @@
       <c r="L30" s="30" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M30" s="30" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="31" t="n">
@@ -1739,6 +1829,9 @@
       <c r="L31" s="31" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M31" s="31" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="32" t="n">
@@ -1777,6 +1870,9 @@
       <c r="L32" s="32" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M32" s="32" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="33" t="n">
@@ -1815,6 +1911,9 @@
       <c r="L33" s="33" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M33" s="33" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="34" t="n">
@@ -1853,6 +1952,9 @@
       <c r="L34" s="34" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M34" s="34" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="35" t="n">
@@ -1891,6 +1993,9 @@
       <c r="L35" s="35" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M35" s="35" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="36" t="n">
@@ -1929,6 +2034,9 @@
       <c r="L36" s="36" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M36" s="36" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="37" t="n">
@@ -1967,6 +2075,9 @@
       <c r="L37" s="37" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M37" s="37" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="38" t="n">
@@ -2005,6 +2116,9 @@
       <c r="L38" s="38" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M38" s="38" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="39" t="n">
@@ -2043,6 +2157,9 @@
       <c r="L39" s="39" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M39" s="39" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="40" t="n">
@@ -2081,6 +2198,9 @@
       <c r="L40" s="40" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M40" s="40" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="41" t="n">
@@ -2119,6 +2239,9 @@
       <c r="L41" s="41" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M41" s="41" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="42" t="n">
@@ -2157,6 +2280,9 @@
       <c r="L42" s="42" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M42" s="42" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="43" t="n">
@@ -2195,6 +2321,9 @@
       <c r="L43" s="43" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M43" s="43" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="44" t="n">
@@ -2233,6 +2362,9 @@
       <c r="L44" s="44" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M44" s="44" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="45" t="n">
@@ -2271,6 +2403,9 @@
       <c r="L45" s="45" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M45" s="45" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="46" t="n">
@@ -2309,6 +2444,9 @@
       <c r="L46" s="46" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M46" s="46" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="17" t="n">
@@ -2347,6 +2485,9 @@
       <c r="L47" s="17" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M47" s="17" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="47" t="n">
@@ -2385,6 +2526,9 @@
       <c r="L48" s="47" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M48" s="47" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="48" t="n">
@@ -2423,6 +2567,9 @@
       <c r="L49" s="48" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M49" s="48" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="17" t="n">
@@ -2461,6 +2608,9 @@
       <c r="L50" s="17" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M50" s="17" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="17" t="n">
@@ -2499,6 +2649,9 @@
       <c r="L51" s="17" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M51" s="17" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="17" t="n">
@@ -2537,6 +2690,9 @@
       <c r="L52" s="17" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M52" s="17" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="25" t="n">
@@ -2575,6 +2731,9 @@
       <c r="L53" s="25" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M53" s="25" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="49" t="n">
@@ -2613,6 +2772,9 @@
       <c r="L54" s="49" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M54" s="49" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="50" t="n">
@@ -2651,6 +2813,9 @@
       <c r="L55" s="50" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M55" s="50" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="17" t="n">
@@ -2689,6 +2854,9 @@
       <c r="L56" s="17" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M56" s="17" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="17" t="n">
@@ -2727,6 +2895,9 @@
       <c r="L57" s="17" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M57" s="17" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="51" t="n">
@@ -2765,6 +2936,9 @@
       <c r="L58" s="51" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M58" s="51" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="52" t="n">
@@ -2803,6 +2977,9 @@
       <c r="L59" s="52" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M59" s="52" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="53" t="n">
@@ -2841,6 +3018,9 @@
       <c r="L60" s="53" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M60" s="53" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="54" t="n">
@@ -2879,6 +3059,9 @@
       <c r="L61" s="54" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M61" s="54" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="55" t="n">
@@ -2917,6 +3100,9 @@
       <c r="L62" s="55" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M62" s="55" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="56" t="n">
@@ -2955,6 +3141,9 @@
       <c r="L63" s="56" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M63" s="56" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="57" t="n">
@@ -2993,6 +3182,9 @@
       <c r="L64" s="57" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M64" s="57" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="58" t="n">
@@ -3031,6 +3223,9 @@
       <c r="L65" s="58" t="n">
         <v>0.999999999</v>
       </c>
+      <c r="M65" s="58" t="n">
+        <v>1E-009</v>
+      </c>
     </row>
     <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="50" t="n">
@@ -3068,6 +3263,9 @@
       </c>
       <c r="L66" s="50" t="n">
         <v>0.999999999</v>
+      </c>
+      <c r="M66" s="50" t="n">
+        <v>1E-009</v>
       </c>
     </row>
   </sheetData>

</xml_diff>